<commit_message>
[update] json 데이터 변경
비어있는 있는 공간 임시로 아무 데이터 삽입
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Enemy.xlsx
+++ b/JsonConverter/ExcelFiles/Enemy.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\JsonConverter\ExcelFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OZ_Project\MinHyeong2DProject\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E6847FD-592E-48F1-A1F5-D063062FB2E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{565333BC-F5EB-4585-8550-9CF0F87E5B88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,9 +30,6 @@
     <t>캐릭터 고유 ID</t>
   </si>
   <si>
-    <t>Id</t>
-  </si>
-  <si>
     <t>enemy_01</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -61,10 +58,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>Reward Gold</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>(name)</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -77,26 +70,14 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>Penalty Life</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>종점 도달 시 깎이는 체력</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>Move Speed</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>Defense</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>Move Type</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>enum</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -121,6 +102,26 @@
   </si>
   <si>
     <t>enemy_05</t>
+  </si>
+  <si>
+    <t>MoveType</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>PenaltyLife</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>RewardGold</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>MoveSpeed</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Id</t>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -572,22 +573,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>8</v>
-      </c>
       <c r="E1" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F1" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="7" t="s">
         <v>14</v>
-      </c>
-      <c r="G1" s="7" t="s">
-        <v>19</v>
       </c>
       <c r="H1" s="7"/>
       <c r="I1" s="7"/>
@@ -596,25 +597,25 @@
     </row>
     <row r="2" spans="1:15" ht="12.75">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
@@ -623,25 +624,25 @@
     </row>
     <row r="3" spans="1:15" s="15" customFormat="1" ht="15.75" customHeight="1">
       <c r="A3" s="13" t="s">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H3" s="14"/>
       <c r="I3" s="14"/>
@@ -650,7 +651,7 @@
     </row>
     <row r="4" spans="1:15" s="17" customFormat="1" ht="15.75" customHeight="1">
       <c r="A4" s="20" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B4" s="21">
         <v>50</v>
@@ -668,7 +669,7 @@
         <v>1</v>
       </c>
       <c r="G4" s="22" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
@@ -681,7 +682,7 @@
     </row>
     <row r="5" spans="1:15" s="17" customFormat="1" ht="15.75" customHeight="1">
       <c r="A5" s="20" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B5" s="20">
         <v>100</v>
@@ -699,7 +700,7 @@
         <v>1</v>
       </c>
       <c r="G5" s="22" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
@@ -712,7 +713,7 @@
     </row>
     <row r="6" spans="1:15" s="17" customFormat="1" ht="15.75" customHeight="1">
       <c r="A6" s="21" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="B6" s="22">
         <v>75</v>
@@ -730,7 +731,7 @@
         <v>1</v>
       </c>
       <c r="G6" s="22" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
@@ -743,7 +744,7 @@
     </row>
     <row r="7" spans="1:15" s="17" customFormat="1" ht="15.75" customHeight="1">
       <c r="A7" s="19" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B7" s="22">
         <v>75</v>
@@ -761,7 +762,7 @@
         <v>1</v>
       </c>
       <c r="G7" s="22" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
@@ -774,7 +775,7 @@
     </row>
     <row r="8" spans="1:15" s="17" customFormat="1" ht="15.75" customHeight="1">
       <c r="A8" s="19" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B8" s="20">
         <v>300</v>
@@ -792,7 +793,7 @@
         <v>2</v>
       </c>
       <c r="G8" s="22" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>

</xml_diff>

<commit_message>
[update] tower_05 구현 및 적 디버프 구현
tower_05 기능 구현 및 적 디버프 구현
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Enemy.xlsx
+++ b/JsonConverter/ExcelFiles/Enemy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OZ_Project\MinHyeong2DProject\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A178715-B738-4A6E-AD14-C1AC3C83244B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1240EA90-879D-4764-BE6C-49B0C1C576B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3855" yWindow="3855" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3240" yWindow="1530" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DNTable_Character&lt;Hero&gt;" sheetId="1" r:id="rId1"/>
@@ -699,7 +699,7 @@
         <v>2.5</v>
       </c>
       <c r="D4" s="22">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E4" s="22">
         <v>50</v>
@@ -732,7 +732,7 @@
         <v>2</v>
       </c>
       <c r="D5" s="22">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E5" s="22">
         <v>75</v>
@@ -765,7 +765,7 @@
         <v>2.5</v>
       </c>
       <c r="D6" s="22">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E6" s="22">
         <v>75</v>
@@ -798,7 +798,7 @@
         <v>3</v>
       </c>
       <c r="D7" s="22">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E7" s="22">
         <v>75</v>
@@ -831,7 +831,7 @@
         <v>1.5</v>
       </c>
       <c r="D8" s="22">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="E8" s="22">
         <v>150</v>

</xml_diff>

<commit_message>
[update] enemy_03, enemy_04, enemy_05 프리팹 생성
enemy_03, enemy_04, enemy_05 프리팹 생성
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Enemy.xlsx
+++ b/JsonConverter/ExcelFiles/Enemy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OZ_Project\MinHyeong2DProject\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1240EA90-879D-4764-BE6C-49B0C1C576B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF239788-BC4C-4F39-8A03-AF08BC745298}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3240" yWindow="1530" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5055" yWindow="2475" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DNTable_Character&lt;Hero&gt;" sheetId="1" r:id="rId1"/>

</xml_diff>